<commit_message>
Update reports 2026-10-07 10:08
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-07.xlsx
+++ b/gex_pivot_levels_2026-10-07.xlsx
@@ -100,19 +100,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -560,33 +560,37 @@
       <c r="G2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="5" t="n">
         <v>7808.57</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="5" t="n">
         <v>7750</v>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>-$9.07M</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>+$18.52M</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>-$9.74M</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>+$19.89M</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -600,14 +604,14 @@
           <t>SPX</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>+$1.20M</t>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$10.57M</t>
+          <t>+$11.26M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -633,7 +637,7 @@
           <t>SPY</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>+$7.45M</t>
         </is>
@@ -664,12 +668,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$13.59M</t>
+          <t>-$13.96M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$22.00M</t>
+          <t>+$22.59M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -695,7 +699,7 @@
           <t>SPY</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>+$7.10M</t>
         </is>
@@ -726,12 +730,12 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>-$809.26K</t>
+          <t>-$818.25K</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>+$35.00M</t>
+          <t>+$35.38M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -753,7 +757,7 @@
           <t>SPX</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>+$4.42M</t>
         </is>
@@ -788,12 +792,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>-$4.76M</t>
+          <t>-$4.71M</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>+$26.18M</t>
+          <t>+$25.93M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -819,14 +823,14 @@
           <t>SPX</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>+$6.39M</t>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>+$6.22M</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>+$50.89M</t>
+          <t>+$49.50M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -848,7 +852,7 @@
           <t>SPY</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>+$24.19M</t>
         </is>
@@ -877,14 +881,14 @@
           <t>SPX</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>+$19.28M</t>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>+$18.29M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$27.02M</t>
+          <t>+$25.62M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -895,66 +899,66 @@
       <c r="G13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="5" t="n">
         <v>7906.7</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="5" t="n">
         <v>782</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>+$41.19M</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>+$41.70M</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="5" t="n">
         <v>7908.57</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="5" t="n">
         <v>7850</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>+$44.52M</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>+$59.36M</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>+$41.74M</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>+$55.65M</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -1024,24 +1028,24 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>31266.53</v>
+        <v>31063.94</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>31030</v>
+        <v>750</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$63.70K</t>
+          <t>-$19.95M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$183.60K</t>
+          <t>+$24.05M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -1053,24 +1057,24 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>31269.46</v>
+        <v>31146.15</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>+$1.97M</t>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>-$12.67M</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>+$14.52M</t>
+          <t>+$20.44M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1082,684 +1086,680 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
+        <v>31266.53</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>31030</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>-$63.70K</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>+$183.60K</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>31269.46</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>755</v>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>-$26.65M</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>+$43.91M</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
         <v>31286.53</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B6" s="2" t="n">
         <v>31050</v>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>-$69.01K</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>+$174.54K</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>31316.53</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <v>31080</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>+$537.69K</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>+$572.66K</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>31336.53</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B8" s="5" t="n">
         <v>31100</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>-$159.24K</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>+$290.39K</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="9">
+      <c r="A9" s="2" t="n">
         <v>31376.53</v>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B9" s="2" t="n">
         <v>31140</v>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>+$19.98K</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>+$149.88K</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="n">
+    <row r="10">
+      <c r="A10" s="5" t="n">
         <v>31386.53</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B10" s="5" t="n">
         <v>31150</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>-$132.70K</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>+$260.10K</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="n">
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>31456.53</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B11" s="5" t="n">
         <v>31220</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>+$595.76K</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>+$764.38K</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="2" t="n">
         <v>31461.53</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B12" s="2" t="n">
         <v>31225</v>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>+$33.72K</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>+$146.13K</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="n">
+    <row r="13">
+      <c r="A13" s="5" t="n">
         <v>31466.53</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B13" s="5" t="n">
         <v>31230</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>+$505.84K</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>+$708.17K</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="n">
+    <row r="14">
+      <c r="A14" s="2" t="n">
         <v>31474.98</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B14" s="2" t="n">
         <v>760</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>+$29.59M</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>+$31.58M</t>
-        </is>
-      </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G12" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>31476.53</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>31240</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>+$11.24K</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>+$258.54K</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>31496.53</v>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>31260</v>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>+$382.19K</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>+$449.63K</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>+$3.65M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$79.67M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
+        <v>31476.53</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>31240</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>+$11.24K</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>+$258.54K</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>31496.53</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>31260</v>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>+$382.19K</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>+$449.63K</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>31511.53</v>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>31275</v>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>-$67.44K</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>+$157.37K</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>31516.08</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>761</v>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>31536.53</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>31300</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>+$202.33K</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>+$550.80K</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>31546.53</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>31310</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>+$84.93K</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$116.78K</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>31557.18</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>762</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>+$3.45M</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>+$4.08M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="n">
-        <v>31536.53</v>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>31300</v>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>+$73.94M</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>+$100.46M</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>31561.53</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>31325</v>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>+$202.33K</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>+$550.80K</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>+$445.89K</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>+$488.35K</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>31546.53</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>31310</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>+$84.93K</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$116.78K</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>31557.18</v>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>762</v>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>+$68.47M</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>+$68.70M</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="n">
-        <v>31561.53</v>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>31325</v>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>+$445.89K</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>+$488.35K</t>
-        </is>
-      </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>31586.53</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>31350</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>+$149.88K</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>+$229.81K</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
+        <v>31586.53</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>31350</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>+$149.88K</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>+$229.81K</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
         <v>31606.53</v>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B23" s="2" t="n">
         <v>31370</v>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>+$4.68K</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>+$70.26K</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
+    <row r="24">
+      <c r="A24" s="5" t="n">
         <v>31636.53</v>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B24" s="5" t="n">
         <v>31400</v>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>+$275.40K</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>+$362.83K</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>31680.49</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>765</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>+$10.53M</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>+$10.83M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G24"/>
@@ -1857,33 +1857,33 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="5" t="n">
         <v>2816.8</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="5" t="n">
         <v>280</v>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>+$3.83M</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>+$13.64M</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -1934,7 +1934,7 @@
           <t>IWM</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>+$4.12M</t>
         </is>
@@ -1967,7 +1967,7 @@
           <t>IWM</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>+$2.09M</t>
         </is>
@@ -1989,33 +1989,33 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="5" t="n">
         <v>2877.16</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <v>286</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>+$6.79M</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>+$6.94M</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -2113,99 +2113,99 @@
       <c r="G2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="5" t="n">
         <v>87.09999999999999</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>-$1.26M</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>+$1.37M</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>88.95999999999999</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>-$38.42K</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>+$1.50M</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="5" t="n">
         <v>90.20999999999999</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="5" t="n">
         <v>145</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>-$2.42M</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>+$4.12M</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -2223,7 +2223,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>+$1.47M</t>
         </is>
@@ -2256,7 +2256,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>+$603.81K</t>
         </is>
@@ -2336,33 +2336,33 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="5" t="n">
         <v>4019.92</v>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="5" t="n">
         <v>85</v>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>-$3.67M</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>+$3.99M</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -2398,33 +2398,33 @@
       <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="5" t="n">
         <v>4114.68</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="5" t="n">
         <v>377</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>-$947.08K</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>+$1.02M</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -2442,7 +2442,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>+$1.24M</t>
         </is>
@@ -2460,33 +2460,33 @@
       <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="5" t="n">
         <v>4161.8</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="5" t="n">
         <v>88</v>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>+$17.29M</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>+$18.70M</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -2504,7 +2504,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>+$1.85M</t>
         </is>
@@ -2537,7 +2537,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>+$147.16K</t>
         </is>
@@ -2570,7 +2570,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>+$803.39K</t>
         </is>
@@ -2592,33 +2592,33 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="5" t="n">
         <v>4202</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="5" t="n">
         <v>385</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>+$2.91M</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>+$3.35M</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -2636,7 +2636,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>+$10.34M</t>
         </is>
@@ -2669,7 +2669,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>+$692.73K</t>
         </is>
@@ -2698,7 +2698,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>+$7.01M</t>
         </is>
@@ -2731,7 +2731,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>+$619.43K</t>
         </is>
@@ -2749,33 +2749,33 @@
       <c r="G14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="5" t="n">
         <v>4280.03</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="5" t="n">
         <v>90.5</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>+$13.08M</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>+$13.17M</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -2793,7 +2793,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>+$47.92K</t>
         </is>
@@ -2815,33 +2815,33 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="5" t="n">
         <v>4350.97</v>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>+$6.71M</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>+$6.89M</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -2916,258 +2916,258 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="5" t="n">
         <v>31557.18</v>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2" s="5" t="n">
         <v>762</v>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>+$68.47M</t>
-        </is>
-      </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>+$68.70M</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>+$73.94M</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>+$100.46M</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>31474.98</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>760</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>+$3.65M</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>+$79.67M</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B4" s="5" t="n">
         <v>7908.57</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C4" s="5" t="n">
         <v>7850</v>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>+$44.52M</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>+$59.36M</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>+$41.74M</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>+$55.65M</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B5" s="2" t="n">
         <v>7883.57</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C5" s="2" t="n">
         <v>7825</v>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>+$6.39M</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>+$50.89M</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>+$6.22M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>+$49.50M</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>31269.46</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>755</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>-$26.65M</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>+$43.91M</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <v>7906.7</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C7" s="5" t="n">
         <v>782</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E7" s="9" t="inlineStr">
         <is>
           <t>+$41.19M</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>+$41.70M</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B8" s="2" t="n">
         <v>7858.57</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>7800</v>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>-$809.26K</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>+$35.00M</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>-$818.25K</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>+$35.38M</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>7886.63</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>780</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>+$24.19M</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>+$32.70M</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>31474.98</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>760</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>+$29.59M</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>+$31.58M</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3176,24 +3176,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>7898.57</v>
+        <v>7886.63</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>7840</v>
+        <v>780</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>+$19.28M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>+$24.19M</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>+$27.02M</t>
+          <t>+$32.70M</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -3222,12 +3222,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>-$4.76M</t>
+          <t>-$4.71M</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>+$26.18M</t>
+          <t>+$25.93M</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3248,62 +3248,58 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7848.57</v>
+        <v>7898.57</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7790</v>
+        <v>7840</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-$13.59M</t>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>+$18.29M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$22.00M</t>
+          <t>+$25.62M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>7836.45</v>
+        <v>31063.94</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>775</v>
+        <v>750</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>+$7.45M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>-$19.95M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>+$21.56M</t>
+          <t>+$24.05M</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
@@ -3320,24 +3316,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7863.57</v>
+        <v>7848.57</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>7805</v>
+        <v>7790</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>+$4.42M</t>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>-$13.96M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$19.35M</t>
+          <t>+$22.59M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -3347,7 +3343,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3358,24 +3354,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7856.52</v>
+        <v>7836.45</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>+$7.10M</t>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>+$7.45M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$19.30M</t>
+          <t>+$21.56M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3386,76 +3382,76 @@
       <c r="H14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>4161.8</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>88</v>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>+$17.29M</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>+$18.70M</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>31146.15</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>752</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>-$12.67M</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>+$20.44M</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>7808.57</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>7750</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>-$9.74M</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>+$19.89M</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>7808.57</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>-$9.07M</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>+$18.52M</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3464,58 +3460,62 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>7806.34</v>
+        <v>7863.57</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>772</v>
+        <v>7805</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>-$4.37M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>+$4.42M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>+$14.63M</t>
+          <t>+$19.35M</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>31269.46</v>
+        <v>7856.52</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>755</v>
+        <v>777</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>+$1.97M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+$7.10M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>+$14.52M</t>
+          <t>+$19.30M</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -3526,178 +3526,178 @@
       <c r="H18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4161.8</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>+$17.29M</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>+$18.70M</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>7806.34</v>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>772</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$4.37M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>+$14.63M</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B21" s="5" t="n">
         <v>2816.8</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C21" s="5" t="n">
         <v>280</v>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>+$3.83M</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>+$13.64M</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B22" s="5" t="n">
         <v>4280.03</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C22" s="5" t="n">
         <v>90.5</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>+$13.08M</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>+$13.17M</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>2826.86</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>281</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>-$747.51K</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>+$11.83M</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>31680.49</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>765</v>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>+$10.53M</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>+$10.83M</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>4256.38</v>
+        <v>2826.86</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>90</v>
+        <v>281</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>+$7.01M</t>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>-$747.51K</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>+$10.79M</t>
+          <t>+$11.83M</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
@@ -3728,14 +3728,14 @@
           <t>SPX</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>+$1.20M</t>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>+$1.28M</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>+$10.57M</t>
+          <t>+$11.26M</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
@@ -3756,24 +3756,24 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>4232.74</v>
+        <v>4256.38</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>89.5</v>
+        <v>90</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>+$10.34M</t>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>+$7.01M</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$10.50M</t>
+          <t>+$10.79M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -3783,309 +3783,309 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>4232.74</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>+$10.34M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$10.50M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B27" s="2" t="n">
         <v>2846.98</v>
       </c>
-      <c r="C26" s="2" t="n">
+      <c r="C27" s="2" t="n">
         <v>283</v>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>+$4.12M</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>+$8.86M</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n">
+      <c r="B28" s="5" t="n">
         <v>2877.16</v>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C28" s="5" t="n">
         <v>286</v>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>+$6.79M</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>+$6.94M</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G28" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B29" s="5" t="n">
         <v>4350.97</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C29" s="5" t="n">
         <v>92</v>
       </c>
-      <c r="D28" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="E29" s="9" t="inlineStr">
         <is>
           <t>+$6.71M</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>+$6.89M</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>2857.04</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="2" t="n">
         <v>284</v>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>+$2.09M</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>+$4.13M</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B31" s="5" t="n">
         <v>90.20999999999999</v>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C31" s="5" t="n">
         <v>145</v>
       </c>
-      <c r="D30" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>-$2.42M</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>+$4.12M</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>31516.08</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>761</v>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>+$3.45M</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>+$4.08M</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>4019.92</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>-$3.67M</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>+$3.99M</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n">
-        <v>4019.92</v>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>85</v>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>-$3.67M</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>+$3.99M</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
+      <c r="B33" s="5" t="n">
+        <v>4202</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>385</v>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>+$2.91M</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>+$3.35M</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H32" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>4202</v>
-      </c>
-      <c r="C33" s="6" t="n">
-        <v>385</v>
-      </c>
-      <c r="D33" s="7" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>+$2.91M</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>+$3.35M</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4108,7 +4108,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>+$1.24M</t>
         </is>
@@ -4142,7 +4142,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>+$1.85M</t>
         </is>
@@ -4180,7 +4180,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>+$1.47M</t>
         </is>
@@ -4240,76 +4240,76 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
+      <c r="B38" s="5" t="n">
         <v>88.95999999999999</v>
       </c>
-      <c r="C38" s="6" t="n">
+      <c r="C38" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="D38" s="7" t="inlineStr">
+      <c r="D38" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>-$38.42K</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>+$1.50M</t>
         </is>
       </c>
-      <c r="G38" s="7" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="6" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n">
+      <c r="B39" s="5" t="n">
         <v>87.09999999999999</v>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="C39" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E39" s="7" t="inlineStr">
         <is>
           <t>-$1.26M</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>+$1.37M</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr">
+      <c r="G39" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4332,7 +4332,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
+      <c r="E40" s="8" t="inlineStr">
         <is>
           <t>+$803.39K</t>
         </is>
@@ -4354,38 +4354,38 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n">
+      <c r="B41" s="5" t="n">
         <v>4114.68</v>
       </c>
-      <c r="C41" s="6" t="n">
+      <c r="C41" s="5" t="n">
         <v>377</v>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E41" s="9" t="inlineStr">
+      <c r="E41" s="7" t="inlineStr">
         <is>
           <t>-$947.08K</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
         <is>
           <t>+$1.02M</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4408,7 +4408,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
+      <c r="E42" s="8" t="inlineStr">
         <is>
           <t>+$692.73K</t>
         </is>
@@ -4442,7 +4442,7 @@
           <t>USO</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="E43" s="8" t="inlineStr">
         <is>
           <t>+$603.81K</t>
         </is>
@@ -4494,76 +4494,76 @@
       <c r="H44" s="3" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B45" s="6" t="n">
+      <c r="B45" s="5" t="n">
         <v>31456.53</v>
       </c>
-      <c r="C45" s="6" t="n">
+      <c r="C45" s="5" t="n">
         <v>31220</v>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
         <is>
           <t>+$595.76K</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>+$764.38K</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n">
+      <c r="B46" s="5" t="n">
         <v>31466.53</v>
       </c>
-      <c r="C46" s="6" t="n">
+      <c r="C46" s="5" t="n">
         <v>31230</v>
       </c>
-      <c r="D46" s="7" t="inlineStr">
+      <c r="D46" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E46" s="9" t="inlineStr">
         <is>
           <t>+$505.84K</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>+$708.17K</t>
         </is>
       </c>
-      <c r="G46" s="7" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4586,7 +4586,7 @@
           <t>GLD</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="E47" s="8" t="inlineStr">
         <is>
           <t>+$619.43K</t>
         </is>
@@ -4604,76 +4604,76 @@
       <c r="H47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B48" s="6" t="n">
+      <c r="B48" s="5" t="n">
         <v>31316.53</v>
       </c>
-      <c r="C48" s="6" t="n">
+      <c r="C48" s="5" t="n">
         <v>31080</v>
       </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E48" s="9" t="inlineStr">
         <is>
           <t>+$537.69K</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
+      <c r="F48" s="6" t="inlineStr">
         <is>
           <t>+$572.66K</t>
         </is>
       </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="G48" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
+      <c r="A49" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B49" s="6" t="n">
+      <c r="B49" s="5" t="n">
         <v>31536.53</v>
       </c>
-      <c r="C49" s="6" t="n">
+      <c r="C49" s="5" t="n">
         <v>31300</v>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E49" s="8" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
         <is>
           <t>+$202.33K</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
         <is>
           <t>+$550.80K</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr">
+      <c r="G49" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4714,114 +4714,114 @@
       <c r="H50" s="3" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B51" s="6" t="n">
+      <c r="B51" s="5" t="n">
         <v>31561.53</v>
       </c>
-      <c r="C51" s="6" t="n">
+      <c r="C51" s="5" t="n">
         <v>31325</v>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E51" s="8" t="inlineStr">
+      <c r="E51" s="9" t="inlineStr">
         <is>
           <t>+$445.89K</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
         <is>
           <t>+$488.35K</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="7" t="inlineStr">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B52" s="6" t="n">
+      <c r="B52" s="5" t="n">
         <v>31496.53</v>
       </c>
-      <c r="C52" s="6" t="n">
+      <c r="C52" s="5" t="n">
         <v>31260</v>
       </c>
-      <c r="D52" s="7" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E52" s="8" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
         <is>
           <t>+$382.19K</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>+$449.63K</t>
         </is>
       </c>
-      <c r="G52" s="7" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H52" s="7" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n">
+      <c r="B53" s="5" t="n">
         <v>31636.53</v>
       </c>
-      <c r="C53" s="6" t="n">
+      <c r="C53" s="5" t="n">
         <v>31400</v>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E53" s="8" t="inlineStr">
+      <c r="E53" s="9" t="inlineStr">
         <is>
           <t>+$275.40K</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>+$362.83K</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4844,7 +4844,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="E54" s="5" t="inlineStr">
+      <c r="E54" s="8" t="inlineStr">
         <is>
           <t>+$147.16K</t>
         </is>
@@ -4866,76 +4866,76 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="7" t="inlineStr">
+      <c r="A55" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n">
+      <c r="B55" s="5" t="n">
         <v>31336.53</v>
       </c>
-      <c r="C55" s="6" t="n">
+      <c r="C55" s="5" t="n">
         <v>31100</v>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E55" s="7" t="inlineStr">
         <is>
           <t>-$159.24K</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
         <is>
           <t>+$290.39K</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr">
+      <c r="G55" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="7" t="inlineStr">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B56" s="6" t="n">
+      <c r="B56" s="5" t="n">
         <v>31386.53</v>
       </c>
-      <c r="C56" s="6" t="n">
+      <c r="C56" s="5" t="n">
         <v>31150</v>
       </c>
-      <c r="D56" s="7" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E56" s="9" t="inlineStr">
+      <c r="E56" s="7" t="inlineStr">
         <is>
           <t>-$132.70K</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>+$260.10K</t>
         </is>
       </c>
-      <c r="G56" s="7" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H56" s="7" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4958,7 +4958,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="E57" s="8" t="inlineStr">
         <is>
           <t>+$11.24K</t>
         </is>
@@ -4996,7 +4996,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E58" s="5" t="inlineStr">
+      <c r="E58" s="8" t="inlineStr">
         <is>
           <t>+$149.88K</t>
         </is>
@@ -5136,7 +5136,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E62" s="5" t="inlineStr">
+      <c r="E62" s="8" t="inlineStr">
         <is>
           <t>+$19.98K</t>
         </is>
@@ -5174,7 +5174,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="E63" s="8" t="inlineStr">
         <is>
           <t>+$33.72K</t>
         </is>
@@ -5212,7 +5212,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E64" s="5" t="inlineStr">
+      <c r="E64" s="8" t="inlineStr">
         <is>
           <t>+$84.93K</t>
         </is>
@@ -5250,7 +5250,7 @@
           <t>GDX</t>
         </is>
       </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="E65" s="8" t="inlineStr">
         <is>
           <t>+$47.92K</t>
         </is>
@@ -5288,7 +5288,7 @@
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
+      <c r="E66" s="8" t="inlineStr">
         <is>
           <t>+$4.68K</t>
         </is>

</xml_diff>